<commit_message>
feat(hardware): align component catalogue with real college lab electronics and web-sourced photos
</commit_message>
<xml_diff>
--- a/public/data/labtrack_master_data.xlsx
+++ b/public/data/labtrack_master_data.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Labs" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Users" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stock" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Projects" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project_Members" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Labs" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Users" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Items" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Stock" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Assets" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Projects" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Project_Members" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -4870,7 +4870,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I35"/>
+  <dimension ref="A1:I40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4879,9 +4879,9 @@
     <col width="25" customWidth="1" min="4" max="4"/>
     <col width="27" customWidth="1" min="5" max="5"/>
     <col width="83" customWidth="1" min="6" max="6"/>
-    <col width="53" customWidth="1" min="7" max="7"/>
+    <col width="58" customWidth="1" min="7" max="7"/>
     <col width="23" customWidth="1" min="8" max="8"/>
-    <col width="41" customWidth="1" min="9" max="9"/>
+    <col width="43" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -5209,7 +5209,7 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>/images/hardware/oscilloscope.jpg</t>
+          <t>/images/hardware/turtlebot-robot.jpg</t>
         </is>
       </c>
     </row>
@@ -5444,7 +5444,7 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>/images/hardware/oscilloscope.jpg</t>
+          <t>/images/hardware/relay-module.jpg</t>
         </is>
       </c>
     </row>
@@ -5498,12 +5498,12 @@
     <row r="14" ht="20" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>WKS-MAC-01</t>
+          <t>MET-DIG-01</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Apple iMac 24" M3 Workstation (16GB / 512GB)</t>
+          <t>Digital Multimeter MAS830L with Test Leads</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -5513,44 +5513,44 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Microprocessors</t>
+          <t>Misc</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Apple Inc.</t>
+          <t>Mastech</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Apple M3 8-core CPU / 10-core GPU, 16GB Unified RAM, 4.5K Retina</t>
+          <t>DC/AC voltage, DC current, resistance, diode test &amp; continuity buzzer</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>High-throughput computer vision workstation</t>
+          <t>Handheld digital circuit measurement instrument</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>Tier 4 High Value</t>
+          <t>Tier 1 Standard</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>/images/hardware/oscilloscope.jpg</t>
+          <t>/images/hardware/digital-multimeter.jpg</t>
         </is>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>WKS-RTX-01</t>
+          <t>CAM-FLI-01</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Dell Precision Tower (NVIDIA RTX 4090 24GB)</t>
+          <t>FLIR Lepton 3.5 Radiometric LWIR Thermal Camera</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -5560,44 +5560,44 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Microprocessors</t>
+          <t>Sensors</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Dell Technologies</t>
+          <t>Teledyne FLIR</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Intel Core i9-14900K, 64GB DDR5, NVIDIA RTX 4090 24GB GDDR6X</t>
+          <t>160x120 thermal resolution, calibrated radiometric temperature output</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Deep learning training workstation</t>
+          <t>Infrared thermal imaging analysis module</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>Tier 4 High Value</t>
+          <t>Tier 3 Advanced</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>/images/hardware/oscilloscope.jpg</t>
+          <t>/images/hardware/realsense-camera.jpg</t>
         </is>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>CAM-FLI-01</t>
+          <t>DIS-OLD-01</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>FLIR Lepton 3.5 Radiometric LWIR Thermal Camera</t>
+          <t>0.96" I2C OLED Display Module (128x64)</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -5607,44 +5607,44 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Sensors</t>
+          <t>Misc</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Teledyne FLIR</t>
+          <t>Solomon Systech</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>160x120 thermal resolution, calibrated radiometric temperature output</t>
+          <t>128x64 pixels, monochrome blue, SSD1306 driver, I2C interface</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Infrared thermal imaging analysis module</t>
+          <t>High contrast graphical status readout display</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>Tier 3 Advanced</t>
+          <t>Tier 1 Standard</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>/images/hardware/realsense-camera.jpg</t>
+          <t>/images/hardware/oled-display.jpg</t>
         </is>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>SEN-UST-01</t>
+          <t>SEN-DHT-01</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Ultrasonic Distance Sensor HC-SR04</t>
+          <t>DHT11 Digital Temperature &amp; Humidity Sensor</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -5659,17 +5659,17 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>ElecFreaks</t>
+          <t>Aosong Electronics</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>2cm to 400cm range, 5V DC, 15-deg measuring angle</t>
+          <t>0 to 50 deg C (+/-2C), 20-90% RH (+/-5% RH), single-wire digital</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Standard sonar distance ranging sensor</t>
+          <t>Cost-effective ambient temperature and humidity sensor</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
@@ -5679,19 +5679,19 @@
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>/images/hardware/bmp280-sensor.jpg</t>
+          <t>/images/hardware/dht11-sensor.jpg</t>
         </is>
       </c>
     </row>
     <row r="18" ht="20" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>SEN-DHT-01</t>
+          <t>SEN-UST-01</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>DHT22 Digital Temperature &amp; Humidity Sensor</t>
+          <t>Ultrasonic Distance Sensor HC-SR04</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -5706,17 +5706,17 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Aosong Electronics</t>
+          <t>ElecFreaks</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>-40 to 80 deg C (+/-0.5C), 0-100% RH (+/-2% RH), single bus</t>
+          <t>2cm to 400cm range, 5V DC, 15-deg measuring angle</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Precision ambient environmental sensor</t>
+          <t>Standard sonar distance ranging sensor</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
@@ -5726,19 +5726,19 @@
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>/images/hardware/bmp280-sensor.jpg</t>
+          <t>/images/hardware/hcsr04-ultrasonic.jpg</t>
         </is>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>SEN-IMU-01</t>
+          <t>SEN-PIR-01</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>MPU6050 6-Axis Gyro &amp; Accelerometer Module</t>
+          <t>PIR Motion Sensor Module HC-SR501</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -5753,17 +5753,17 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>TDK InvenSense</t>
+          <t>ElecFreaks</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>3-axis gyro (+/-2000 dps), 3-axis accel (+/-16g), I2C interface</t>
+          <t>3m to 7m range, 100-deg cone, 5V-20V DC, adjustable trigger</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Motion tracking inertial measurement unit</t>
+          <t>Passive infrared motion detection module</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
@@ -5773,19 +5773,19 @@
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>/images/hardware/bmp280-sensor.jpg</t>
+          <t>/images/hardware/pir-motion-sensor.jpg</t>
         </is>
       </c>
     </row>
     <row r="20" ht="20" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>SEN-BMP-01</t>
+          <t>SEN-IRS-01</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>BMP280 Barometric Pressure Sensor</t>
+          <t>Infrared Obstacle Avoidance Sensor Module</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -5800,17 +5800,17 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Bosch Sensortec</t>
+          <t>Waveshare</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>300 to 1100 hPa (+/-1 hPa), I2C/SPI interface, 3.3V</t>
+          <t>2cm to 30cm detection range, 35-deg angle, LM393 comparator</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Altimeter and atmospheric pressure module</t>
+          <t>Active infrared proximity and obstacle detector</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
@@ -5820,19 +5820,19 @@
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>/images/hardware/bmp280-sensor.jpg</t>
+          <t>/images/hardware/ir-sensor-module.jpg</t>
         </is>
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>SEN-LIN-01</t>
+          <t>SEN-PZO-01</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>TCRT5000 5-Channel Infrared Line Tracking Array</t>
+          <t>Piezoelectric Vibration &amp; Knock Sensor</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -5847,17 +5847,17 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Waveshare</t>
+          <t>Generic</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>5-channel reflective optical sensor, digital output, adjustable sensitivity</t>
+          <t>Ceramic piezo disc 27mm, analog voltage output proportional to impact</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>Robotics line-following tracker board</t>
+          <t>Vibration, knock, and shock detection disc</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
@@ -5867,19 +5867,19 @@
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>/images/hardware/bmp280-sensor.jpg</t>
+          <t>/images/hardware/piezo-sensor.jpg</t>
         </is>
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>MCU-UNO-01</t>
+          <t>SEN-BMP-01</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Arduino Uno Rev3 DIP Microcontroller</t>
+          <t>BMP280 Barometric Pressure Sensor</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -5889,22 +5889,22 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Microcontrollers</t>
+          <t>Sensors</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Arduino LLC</t>
+          <t>Bosch Sensortec</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>ATmega328P 16MHz, 32KB Flash, 14 Digital IO, 6 PWM, 6 ADC</t>
+          <t>300 to 1100 hPa (+/-1 hPa), I2C/SPI interface, 3.3V</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Standard prototyping microcontroller platform</t>
+          <t>Altimeter and atmospheric pressure module</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
@@ -5914,19 +5914,19 @@
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>/images/hardware/arduino-uno-r3.jpg</t>
+          <t>/images/hardware/bmp280-sensor.jpg</t>
         </is>
       </c>
     </row>
     <row r="23" ht="20" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>MCU-ESP-01</t>
+          <t>SEN-IMU-01</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>ESP32-WROOM-32 Wi-Fi + BLE Development Board</t>
+          <t>MPU6050 6-Axis Gyro &amp; Accelerometer Module</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -5936,22 +5936,22 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Microcontrollers</t>
+          <t>Sensors</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Espressif Systems</t>
+          <t>TDK InvenSense</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Dual-core Xtensa 32-bit LX6 @ 240MHz, 802.11 b/g/n, Bluetooth v4.2 BR/EDR &amp; BLE</t>
+          <t>3-axis gyro (+/-2000 dps), 3-axis accel (+/-16g), I2C interface</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>High-performance IoT controller</t>
+          <t>Motion tracking inertial measurement unit</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
@@ -5961,19 +5961,19 @@
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>/images/hardware/esp32-wroom.jpg</t>
+          <t>/images/hardware/bmp280-sensor.jpg</t>
         </is>
       </c>
     </row>
     <row r="24" ht="20" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>MCU-RP2-01</t>
+          <t>SEN-LIN-01</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Raspberry Pi Pico W</t>
+          <t>TCRT5000 5-Channel Infrared Line Tracking Array</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -5983,22 +5983,22 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Microcontrollers</t>
+          <t>Sensors</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Raspberry Pi Foundation</t>
+          <t>Waveshare</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>RP2040 Dual-core ARM Cortex-M0+ @ 133MHz, Infineon CYW43439 Wi-Fi 4</t>
+          <t>5-channel reflective optical sensor, digital output, adjustable sensitivity</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>Low cost wireless micro-controller</t>
+          <t>Robotics line-following tracker board</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
@@ -6008,19 +6008,19 @@
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>/images/hardware/arduino-uno-r3.jpg</t>
+          <t>/images/hardware/ir-sensor-module.jpg</t>
         </is>
       </c>
     </row>
     <row r="25" ht="20" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>COM-GPS-01</t>
+          <t>MCU-UNO-01</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>U-Blox Neo-6M GPS Module with Active Antenna</t>
+          <t>Arduino Uno Rev3 DIP Microcontroller</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -6030,22 +6030,22 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Communication Modules</t>
+          <t>Microcontrollers</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>u-blox</t>
+          <t>Arduino LLC</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>50-channel GPS engine, UART TTL output, EEPROM backup, PPS indicator</t>
+          <t>ATmega328P 16MHz, 32KB Flash, 14 Digital IO, 6 PWM, 6 ADC</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>Satellite navigation and positioning module</t>
+          <t>Standard prototyping microcontroller platform</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
@@ -6055,19 +6055,19 @@
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>/images/hardware/esp32-wroom.jpg</t>
+          <t>/images/hardware/arduino-uno-r3.jpg</t>
         </is>
       </c>
     </row>
     <row r="26" ht="20" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>COM-NRF-01</t>
+          <t>MCU-ESP-01</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>nRF24L01+ 2.4GHz Wireless RF Transceiver</t>
+          <t>ESP32-WROOM-32 Wi-Fi + BLE Development Board</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -6077,22 +6077,22 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Communication Modules</t>
+          <t>Microcontrollers</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Nordic Semiconductor</t>
+          <t>Espressif Systems</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>2.4GHz ISM band, 250kbps to 2Mbps, SPI interface, ultra low power</t>
+          <t>Dual-core Xtensa 32-bit LX6 @ 240MHz, 802.11 b/g/n, Bluetooth v4.2 BR/EDR &amp; BLE</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Wireless point-to-point data telemetry link</t>
+          <t>High-performance IoT controller</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
@@ -6109,12 +6109,12 @@
     <row r="27" ht="20" customHeight="1">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>MOT-SRV-01</t>
+          <t>MCU-RP2-01</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>TowerPro SG90 9g Micro Servo Motor</t>
+          <t>Raspberry Pi Pico W</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -6124,22 +6124,22 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Motors</t>
+          <t>Microcontrollers</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>TowerPro</t>
+          <t>Raspberry Pi Foundation</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>180-degree rotation, 1.8 kg-cm torque @ 4.8V, nylon gears</t>
+          <t>RP2040 Dual-core ARM Cortex-M0+ @ 133MHz, Infineon CYW43439 Wi-Fi 4</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>Lightweight robotic steering &amp; pan-tilt servo</t>
+          <t>Low cost wireless micro-controller</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
@@ -6149,19 +6149,19 @@
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>/images/hardware/breadboard-830.jpg</t>
+          <t>/images/hardware/arduino-uno-r3.jpg</t>
         </is>
       </c>
     </row>
     <row r="28" ht="20" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>MOT-SRV-02</t>
+          <t>COM-GPS-01</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>MG996R High Torque Metal Gear Servo Motor</t>
+          <t>U-Blox Neo-6M GPS Module with Active Antenna</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -6171,22 +6171,22 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Motors</t>
+          <t>Communication Modules</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>TowerPro</t>
+          <t>u-blox</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>180-degree rotation, 11 kg-cm torque @ 6V, all metal gear train</t>
+          <t>50-channel GPS engine, UART TTL output, EEPROM backup, PPS indicator</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Heavy duty robotic joint actuator</t>
+          <t>Satellite navigation and positioning module</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
@@ -6196,19 +6196,19 @@
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>/images/hardware/breadboard-830.jpg</t>
+          <t>/images/hardware/esp32-wroom.jpg</t>
         </is>
       </c>
     </row>
     <row r="29" ht="20" customHeight="1">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>MOT-STP-01</t>
+          <t>COM-NRF-01</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>NEMA 17 Bipolar Stepper Motor (1.5A 42mm)</t>
+          <t>nRF24L01+ 2.4GHz Wireless RF Transceiver</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
@@ -6218,22 +6218,22 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Motors</t>
+          <t>Communication Modules</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>StepperOnline</t>
+          <t>Nordic Semiconductor</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>1.8 deg step angle (200 steps/rev), 45 Ncm holding torque, 4-wire lead</t>
+          <t>2.4GHz ISM band, 250kbps to 2Mbps, SPI interface, ultra low power</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>Precision CNC and 3D printing drive motor</t>
+          <t>Wireless point-to-point data telemetry link</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -6243,19 +6243,19 @@
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>/images/hardware/breadboard-830.jpg</t>
+          <t>/images/hardware/esp32-wroom.jpg</t>
         </is>
       </c>
     </row>
     <row r="30" ht="20" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>DRV-MOT-01</t>
+          <t>MOT-SRV-01</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>L298N Dual H-Bridge Motor Driver Module</t>
+          <t>TowerPro SG90 9g Micro Servo Motor</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -6270,17 +6270,17 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>STMicroelectronics</t>
+          <t>TowerPro</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Dual 2A H-bridge driver, 5V to 35V drive voltage, opto-isolated</t>
+          <t>180-degree rotation, 1.8 kg-cm torque @ 4.8V, nylon gears</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Dual DC motor and stepper motor driver</t>
+          <t>Lightweight robotic steering &amp; pan-tilt servo</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -6290,19 +6290,19 @@
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>/images/hardware/breadboard-830.jpg</t>
+          <t>/images/hardware/sg90-servo.jpg</t>
         </is>
       </c>
     </row>
     <row r="31" ht="20" customHeight="1">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>PWR-LIP-01</t>
+          <t>MOT-SRV-02</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>11.1V 3S LiPo Battery Pack 2200mAh 30C</t>
+          <t>MG996R High Torque Metal Gear Servo Motor</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
@@ -6312,22 +6312,22 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Batteries</t>
+          <t>Motors</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Orange Power</t>
+          <t>TowerPro</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>3S1P 11.1V, 2200mAh capacity, 30C discharge, XT60 connector</t>
+          <t>180-degree rotation, 11 kg-cm torque @ 6V, all metal gear train</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>High discharge battery pack for mobile robots</t>
+          <t>Heavy duty robotic joint actuator</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
@@ -6337,19 +6337,19 @@
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>/images/hardware/breadboard-830.jpg</t>
+          <t>/images/hardware/sg90-servo.jpg</t>
         </is>
       </c>
     </row>
     <row r="32" ht="20" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>PWR-ION-01</t>
+          <t>MOT-STP-01</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Samsung 18650 Li-ion Cell 3.7V 2600mAh</t>
+          <t>NEMA 17 Bipolar Stepper Motor (1.5A 42mm)</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -6359,22 +6359,22 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Batteries</t>
+          <t>Motors</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Samsung SDI</t>
+          <t>StepperOnline</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>3.7V nominal, 2600mAh capacity, rechargeable flat-top cylindrical cell</t>
+          <t>1.8 deg step angle (200 steps/rev), 45 Ncm holding torque, 4-wire lead</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Standard rechargeable power cell for field nodes</t>
+          <t>Precision CNC and 3D printing drive motor</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
@@ -6384,19 +6384,19 @@
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>/images/hardware/breadboard-830.jpg</t>
+          <t>/images/hardware/nema17-stepper.jpg</t>
         </is>
       </c>
     </row>
     <row r="33" ht="20" customHeight="1">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>PRT-BRD-01</t>
+          <t>DRV-MOT-01</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>830-Tie Point Solderless Breadboard</t>
+          <t>L298N Dual H-Bridge Motor Driver Module</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
@@ -6406,22 +6406,22 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Misc</t>
+          <t>Motors</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>Generic High Quality</t>
+          <t>STMicroelectronics</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>830 tie points (630 IC points + 200 power bus rails), standard 2.54mm pitch</t>
+          <t>Dual 2A H-bridge driver, 5V to 35V drive voltage, opto-isolated</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>Solderless electronic circuit prototype board</t>
+          <t>Dual DC motor and stepper motor driver</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
@@ -6431,19 +6431,19 @@
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>/images/hardware/breadboard-830.jpg</t>
+          <t>/images/hardware/l298n-motor-driver.jpg</t>
         </is>
       </c>
     </row>
     <row r="34" ht="20" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>PRT-JMP-01</t>
+          <t>PWR-9VB-01</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>40-Pin Multi-Color Jumper Wires (M-to-F 20cm)</t>
+          <t>9V Heavy Duty Alkaline Battery</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -6453,22 +6453,22 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Misc</t>
+          <t>Batteries</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Generic</t>
+          <t>Hi-Watt / Duracell</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>40-conductor ribbon cable, Male-to-Female 2.54mm pitch, 20cm length</t>
+          <t>Standard 9V 6F22 primary power cell with snap terminals</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Essential lab circuit prototyping patch wires</t>
+          <t>Portable DC power for microcontrollers and sensors</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
@@ -6478,54 +6478,289 @@
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>/images/hardware/jumper-wires.jpg</t>
+          <t>/images/hardware/9v-battery.jpg</t>
         </is>
       </c>
     </row>
     <row r="35" ht="20" customHeight="1">
       <c r="A35" s="2" t="inlineStr">
         <is>
+          <t>PWR-ION-01</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Samsung 18650 Li-ion Cell 3.7V 2600mAh</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>CONSUMABLE</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Batteries</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>Samsung SDI</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>3.7V nominal, 2600mAh capacity, rechargeable flat-top cylindrical cell</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>Standard rechargeable power cell for field nodes</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>Tier 1 Standard</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t>/images/hardware/18650-battery.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="20" customHeight="1">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>PWR-LIP-01</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>11.1V 3S LiPo Battery Pack 2200mAh 30C</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>CONSUMABLE</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>Batteries</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>Orange Power</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>3S1P 11.1V, 2200mAh capacity, 30C discharge, XT60 connector</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>High discharge battery pack for mobile robots</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>Tier 1 Standard</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>/images/hardware/18650-battery.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="20" customHeight="1">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>PRT-BRD-01</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>830-Tie Point Solderless Breadboard</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>CONSUMABLE</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>Generic High Quality</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>830 tie points (630 IC points + 200 power bus rails), standard 2.54mm pitch</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>Solderless electronic circuit prototype board</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>Tier 1 Standard</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>/images/hardware/breadboard-830.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="20" customHeight="1">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>PRT-JMP-01</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>40-Pin Multi-Color Jumper Wires (M-to-F 20cm)</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>CONSUMABLE</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>Generic</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>40-conductor ribbon cable, Male-to-Female 2.54mm pitch, 20cm length</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>Essential lab circuit prototyping patch wires</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>Tier 1 Standard</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>/images/hardware/jumper-wires.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="20" customHeight="1">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
           <t>RLY-MOD-01</t>
         </is>
       </c>
-      <c r="B35" s="2" t="inlineStr">
+      <c r="B39" s="2" t="inlineStr">
         <is>
           <t>4-Channel 5V Relay Module with Optocoupler</t>
         </is>
       </c>
-      <c r="C35" s="2" t="inlineStr">
+      <c r="C39" s="2" t="inlineStr">
         <is>
           <t>CONSUMABLE</t>
         </is>
       </c>
-      <c r="D35" s="2" t="inlineStr">
+      <c r="D39" s="2" t="inlineStr">
         <is>
           <t>Misc</t>
         </is>
       </c>
-      <c r="E35" s="2" t="inlineStr">
+      <c r="E39" s="2" t="inlineStr">
         <is>
           <t>Songle</t>
         </is>
       </c>
-      <c r="F35" s="2" t="inlineStr">
+      <c r="F39" s="2" t="inlineStr">
         <is>
           <t>4x SPDT 10A 250VAC / 30VDC relays, active low trigger, status LEDs</t>
         </is>
       </c>
-      <c r="G35" s="2" t="inlineStr">
+      <c r="G39" s="2" t="inlineStr">
         <is>
           <t>High-voltage AC/DC circuit switching board</t>
         </is>
       </c>
-      <c r="H35" s="2" t="inlineStr">
+      <c r="H39" s="2" t="inlineStr">
         <is>
           <t>Tier 1 Standard</t>
         </is>
       </c>
-      <c r="I35" s="2" t="inlineStr">
-        <is>
-          <t>/images/hardware/breadboard-830.jpg</t>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>/images/hardware/relay-module.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="20" customHeight="1">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>DIS-LCD-01</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>16x2 Character LCD Display Module</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>CONSUMABLE</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>Misc</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>Hitachi / Generic</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>16 characters x 2 lines, blue backlight, 5V HD44780 controller</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>Alphanumeric character readout display</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>Tier 1 Standard</t>
+        </is>
+      </c>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>/images/hardware/lcd-1602.jpg</t>
         </is>
       </c>
     </row>
@@ -6540,7 +6775,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G56"/>
+  <dimension ref="A1:G68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -6685,32 +6920,32 @@
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>OSTL-CSE</t>
+          <t>PPSL-CSE</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Open Source Tools Lab</t>
+          <t>Programming and Problem Solving Lab</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>SBC-RPI-04</t>
+          <t>PWR-9VB-01</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Raspberry Pi 4 Model B 4GB RAM</t>
+          <t>9V Heavy Duty Alkaline Battery</t>
         </is>
       </c>
       <c r="E5" s="3" t="n">
-        <v>8</v>
+        <v>30</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>9</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
@@ -6726,22 +6961,22 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>MCU-ESP-01</t>
+          <t>SBC-RPI-04</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>ESP32-WROOM-32 Wi-Fi + BLE Development Board</t>
+          <t>Raspberry Pi 4 Model B 4GB RAM</t>
         </is>
       </c>
       <c r="E6" s="3" t="n">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>22</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
@@ -6757,177 +6992,177 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>SEN-UST-01</t>
+          <t>MCU-ESP-01</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Ultrasonic Distance Sensor HC-SR04</t>
+          <t>ESP32-WROOM-32 Wi-Fi + BLE Development Board</t>
         </is>
       </c>
       <c r="E7" s="3" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>16</v>
+        <v>22</v>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>DSL-CSE</t>
+          <t>OSTL-CSE</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Data Structure Lab (CL-06)</t>
+          <t>Open Source Tools Lab</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>MCU-RP2-01</t>
+          <t>SEN-UST-01</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Raspberry Pi Pico W</t>
+          <t>Ultrasonic Distance Sensor HC-SR04</t>
         </is>
       </c>
       <c r="E8" s="3" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>32</v>
+        <v>16</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>DSL-CSE</t>
+          <t>OSTL-CSE</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Data Structure Lab (CL-06)</t>
+          <t>Open Source Tools Lab</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>PRT-BRD-01</t>
+          <t>SEN-IRS-01</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>830-Tie Point Solderless Breadboard</t>
+          <t>Infrared Obstacle Avoidance Sensor Module</t>
         </is>
       </c>
       <c r="E9" s="3" t="n">
-        <v>35</v>
+        <v>20</v>
       </c>
       <c r="F9" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>36</v>
+        <v>21</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>PL-CSE</t>
+          <t>DSL-CSE</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Project Lab (CL-7)</t>
+          <t>Data Structure Lab (CL-06)</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>SBC-RPI-05</t>
+          <t>MCU-RP2-01</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Raspberry Pi 5 Model B 8GB RAM</t>
+          <t>Raspberry Pi Pico W</t>
         </is>
       </c>
       <c r="E10" s="3" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>10</v>
+        <v>32</v>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>PL-CSE</t>
+          <t>DSL-CSE</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Project Lab (CL-7)</t>
+          <t>Data Structure Lab (CL-06)</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>DEV-JET-01</t>
+          <t>PRT-BRD-01</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>NVIDIA Jetson Nano 4GB B01 Developer Kit</t>
+          <t>830-Tie Point Solderless Breadboard</t>
         </is>
       </c>
       <c r="E11" s="3" t="n">
-        <v>6</v>
+        <v>35</v>
       </c>
       <c r="F11" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>7</v>
+        <v>36</v>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>PL-CSE</t>
+          <t>DSL-CSE</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Project Lab (CL-7)</t>
+          <t>Data Structure Lab (CL-06)</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>OSC-RIG-01</t>
+          <t>DIS-LCD-01</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Rigol DS1054Z 50MHz Digital Oscilloscope</t>
+          <t>16x2 Character LCD Display Module</t>
         </is>
       </c>
       <c r="E12" s="3" t="n">
-        <v>3</v>
+        <v>20</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>3</v>
+        <v>21</v>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
@@ -6943,22 +7178,22 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>COM-GPS-01</t>
+          <t>SBC-RPI-05</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>U-Blox Neo-6M GPS Module with Active Antenna</t>
+          <t>Raspberry Pi 5 Model B 8GB RAM</t>
         </is>
       </c>
       <c r="E13" s="3" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F13" s="3" t="n">
         <v>0</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
@@ -6974,281 +7209,281 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>RLY-MOD-01</t>
+          <t>DEV-JET-01</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>4-Channel 5V Relay Module with Optocoupler</t>
+          <t>NVIDIA Jetson Nano 4GB B01 Developer Kit</t>
         </is>
       </c>
       <c r="E14" s="3" t="n">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="F14" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>19</v>
+        <v>7</v>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>DMAL-CSE</t>
+          <t>PL-CSE</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Database Management and Analytics Lab (CL-9)</t>
+          <t>Project Lab (CL-7)</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>SBC-RPI-05</t>
+          <t>OSC-RIG-01</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Raspberry Pi 5 Model B 8GB RAM</t>
+          <t>Rigol DS1054Z 50MHz Digital Oscilloscope</t>
         </is>
       </c>
       <c r="E15" s="3" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="F15" s="3" t="n">
         <v>0</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>DMAL-CSE</t>
+          <t>PL-CSE</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Database Management and Analytics Lab (CL-9)</t>
+          <t>Project Lab (CL-7)</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>SEN-DHT-01</t>
+          <t>COM-GPS-01</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>DHT22 Digital Temperature &amp; Humidity Sensor</t>
+          <t>U-Blox Neo-6M GPS Module with Active Antenna</t>
         </is>
       </c>
       <c r="E16" s="3" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>22</v>
+        <v>12</v>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>MTECH-CSE</t>
+          <t>PL-CSE</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>M.Tech Research Lab</t>
+          <t>Project Lab (CL-7)</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>WKS-RTX-01</t>
+          <t>RLY-MOD-01</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Dell Precision Tower (NVIDIA RTX 4090 24GB)</t>
+          <t>4-Channel 5V Relay Module with Optocoupler</t>
         </is>
       </c>
       <c r="E17" s="3" t="n">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>4</v>
+        <v>19</v>
       </c>
     </row>
     <row r="18" ht="20" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>MTECH-CSE</t>
+          <t>PL-CSE</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>M.Tech Research Lab</t>
+          <t>Project Lab (CL-7)</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>DEV-JET-02</t>
+          <t>SEN-PIR-01</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>NVIDIA Jetson Orin Nano Developer Kit (8GB)</t>
+          <t>PIR Motion Sensor Module HC-SR501</t>
         </is>
       </c>
       <c r="E18" s="3" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>5</v>
+        <v>16</v>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>MTECH-CSE</t>
+          <t>PL-CSE</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>M.Tech Research Lab</t>
+          <t>Project Lab (CL-7)</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>CAM-INT-01</t>
+          <t>DIS-OLD-01</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Intel RealSense Depth Camera D435i</t>
+          <t>0.96" I2C OLED Display Module (128x64)</t>
         </is>
       </c>
       <c r="E19" s="3" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>3</v>
+        <v>16</v>
       </c>
     </row>
     <row r="20" ht="20" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>DV-AIML</t>
+          <t>DMAL-CSE</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Data Visualization Lab (Workstation)</t>
+          <t>Database Management and Analytics Lab (CL-9)</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>WKS-RTX-01</t>
+          <t>SBC-RPI-05</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Dell Precision Tower (NVIDIA RTX 4090 24GB)</t>
+          <t>Raspberry Pi 5 Model B 8GB RAM</t>
         </is>
       </c>
       <c r="E20" s="3" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F20" s="3" t="n">
         <v>0</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>DV-AIML</t>
+          <t>DMAL-CSE</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Data Visualization Lab (Workstation)</t>
+          <t>Database Management and Analytics Lab (CL-9)</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>DEV-JET-01</t>
+          <t>SEN-DHT-01</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>NVIDIA Jetson Nano 4GB B01 Developer Kit</t>
+          <t>DHT11 Digital Temperature &amp; Humidity Sensor</t>
         </is>
       </c>
       <c r="E21" s="3" t="n">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>9</v>
+        <v>22</v>
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>CV-AIML</t>
+          <t>MTECH-CSE</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Computer Vision Lab (iMac Lab)</t>
+          <t>M.Tech Research Lab</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>WKS-MAC-01</t>
+          <t>DEV-JET-02</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Apple iMac 24" M3 Workstation (16GB / 512GB)</t>
+          <t>NVIDIA Jetson Orin Nano Developer Kit (8GB)</t>
         </is>
       </c>
       <c r="E22" s="3" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="F22" s="3" t="n">
         <v>0</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
     </row>
     <row r="23" ht="20" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>CV-AIML</t>
+          <t>MTECH-CSE</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Computer Vision Lab (iMac Lab)</t>
+          <t>M.Tech Research Lab</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -7262,34 +7497,34 @@
         </is>
       </c>
       <c r="E23" s="3" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F23" s="3" t="n">
         <v>0</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="24" ht="20" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>CV-AIML</t>
+          <t>MTECH-CSE</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Computer Vision Lab (iMac Lab)</t>
+          <t>M.Tech Research Lab</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>CAM-FLI-01</t>
+          <t>MET-DIG-01</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>FLIR Lepton 3.5 Radiometric LWIR Thermal Camera</t>
+          <t>Digital Multimeter MAS830L with Test Leads</t>
         </is>
       </c>
       <c r="E24" s="3" t="n">
@@ -7305,992 +7540,1364 @@
     <row r="25" ht="20" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>MDL-AIML</t>
+          <t>DV-AIML</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Machine and Deep Learning Lab</t>
+          <t>Data Visualization Lab (Workstation)</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>DEV-JET-02</t>
+          <t>DEV-JET-01</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>NVIDIA Jetson Orin Nano Developer Kit (8GB)</t>
+          <t>NVIDIA Jetson Nano 4GB B01 Developer Kit</t>
         </is>
       </c>
       <c r="E25" s="3" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="26" ht="20" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>MDL-AIML</t>
+          <t>DV-AIML</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Machine and Deep Learning Lab</t>
+          <t>Data Visualization Lab (Workstation)</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>DEV-JET-01</t>
+          <t>MET-DIG-01</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>NVIDIA Jetson Nano 4GB B01 Developer Kit</t>
+          <t>Digital Multimeter MAS830L with Test Leads</t>
         </is>
       </c>
       <c r="E26" s="3" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>14</v>
+        <v>6</v>
       </c>
     </row>
     <row r="27" ht="20" customHeight="1">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>MDL-AIML</t>
+          <t>CV-AIML</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Machine and Deep Learning Lab</t>
+          <t>Computer Vision Lab (iMac Lab)</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>SEN-IMU-01</t>
+          <t>CAM-INT-01</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>MPU6050 6-Axis Gyro &amp; Accelerometer Module</t>
+          <t>Intel RealSense Depth Camera D435i</t>
         </is>
       </c>
       <c r="E27" s="3" t="n">
-        <v>25</v>
+        <v>6</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>28</v>
+        <v>6</v>
       </c>
     </row>
     <row r="28" ht="20" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>NLP-AIML</t>
+          <t>CV-AIML</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Natural Language Processing Lab</t>
+          <t>Computer Vision Lab (iMac Lab)</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>SBC-RPI-05</t>
+          <t>CAM-FLI-01</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Raspberry Pi 5 Model B 8GB RAM</t>
+          <t>FLIR Lepton 3.5 Radiometric LWIR Thermal Camera</t>
         </is>
       </c>
       <c r="E28" s="3" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
     </row>
     <row r="29" ht="20" customHeight="1">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>NLP-AIML</t>
+          <t>CV-AIML</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Natural Language Processing Lab</t>
+          <t>Computer Vision Lab (iMac Lab)</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>MCU-ESP-01</t>
+          <t>MET-DIG-01</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>ESP32-WROOM-32 Wi-Fi + BLE Development Board</t>
+          <t>Digital Multimeter MAS830L with Test Leads</t>
         </is>
       </c>
       <c r="E29" s="3" t="n">
-        <v>30</v>
+        <v>12</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>32</v>
+        <v>12</v>
       </c>
     </row>
     <row r="30" ht="20" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>CCL-AIML</t>
+          <t>MDL-AIML</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Cloud Computing Lab</t>
+          <t>Machine and Deep Learning Lab</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>DEV-JET-01</t>
+          <t>DEV-JET-02</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>NVIDIA Jetson Nano 4GB B01 Developer Kit</t>
+          <t>NVIDIA Jetson Orin Nano Developer Kit (8GB)</t>
         </is>
       </c>
       <c r="E30" s="3" t="n">
         <v>10</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="31" ht="20" customHeight="1">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>CCL-AIML</t>
+          <t>MDL-AIML</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Cloud Computing Lab</t>
+          <t>Machine and Deep Learning Lab</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>SBC-RPI-04</t>
+          <t>DEV-JET-01</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Raspberry Pi 4 Model B 4GB RAM</t>
+          <t>NVIDIA Jetson Nano 4GB B01 Developer Kit</t>
         </is>
       </c>
       <c r="E31" s="3" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="F31" s="3" t="n">
         <v>2</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="32" ht="20" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>CCL-AIML</t>
+          <t>MDL-AIML</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Cloud Computing Lab</t>
+          <t>Machine and Deep Learning Lab</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>MCU-ESP-01</t>
+          <t>SEN-IMU-01</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>ESP32-WROOM-32 Wi-Fi + BLE Development Board</t>
+          <t>MPU6050 6-Axis Gyro &amp; Accelerometer Module</t>
         </is>
       </c>
       <c r="E32" s="3" t="n">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="F32" s="3" t="n">
         <v>3</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>38</v>
+        <v>28</v>
       </c>
     </row>
     <row r="33" ht="20" customHeight="1">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>CCL-AIML</t>
+          <t>NLP-AIML</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Cloud Computing Lab</t>
+          <t>Natural Language Processing Lab</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>SEN-BMP-01</t>
+          <t>SBC-RPI-05</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>BMP280 Barometric Pressure Sensor</t>
+          <t>Raspberry Pi 5 Model B 8GB RAM</t>
         </is>
       </c>
       <c r="E33" s="3" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="F33" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>21</v>
+        <v>13</v>
       </c>
     </row>
     <row r="34" ht="20" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>MSA-AIML</t>
+          <t>NLP-AIML</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Multimodal Sensor Analytics Lab</t>
+          <t>Natural Language Processing Lab</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>SEN-UST-01</t>
+          <t>MCU-ESP-01</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Ultrasonic Distance Sensor HC-SR04</t>
+          <t>ESP32-WROOM-32 Wi-Fi + BLE Development Board</t>
         </is>
       </c>
       <c r="E34" s="3" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>44</v>
+        <v>32</v>
       </c>
     </row>
     <row r="35" ht="20" customHeight="1">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>MSA-AIML</t>
+          <t>CCL-AIML</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Multimodal Sensor Analytics Lab</t>
+          <t>Cloud Computing Lab</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>SEN-DHT-01</t>
+          <t>DEV-JET-01</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>DHT22 Digital Temperature &amp; Humidity Sensor</t>
+          <t>NVIDIA Jetson Nano 4GB B01 Developer Kit</t>
         </is>
       </c>
       <c r="E35" s="3" t="n">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>37</v>
+        <v>11</v>
       </c>
     </row>
     <row r="36" ht="20" customHeight="1">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>MSA-AIML</t>
+          <t>CCL-AIML</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Multimodal Sensor Analytics Lab</t>
+          <t>Cloud Computing Lab</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>SEN-IMU-01</t>
+          <t>SBC-RPI-04</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>MPU6050 6-Axis Gyro &amp; Accelerometer Module</t>
+          <t>Raspberry Pi 4 Model B 4GB RAM</t>
         </is>
       </c>
       <c r="E36" s="3" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="F36" s="3" t="n">
         <v>2</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>32</v>
+        <v>17</v>
       </c>
     </row>
     <row r="37" ht="20" customHeight="1">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>MSA-AIML</t>
+          <t>CCL-AIML</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Multimodal Sensor Analytics Lab</t>
+          <t>Cloud Computing Lab</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>SEN-BMP-01</t>
+          <t>MCU-ESP-01</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>BMP280 Barometric Pressure Sensor</t>
+          <t>ESP32-WROOM-32 Wi-Fi + BLE Development Board</t>
         </is>
       </c>
       <c r="E37" s="3" t="n">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>26</v>
+        <v>38</v>
       </c>
     </row>
     <row r="38" ht="20" customHeight="1">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>MSA-AIML</t>
+          <t>CCL-AIML</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Multimodal Sensor Analytics Lab</t>
+          <t>Cloud Computing Lab</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>COM-GPS-01</t>
+          <t>SEN-BMP-01</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>U-Blox Neo-6M GPS Module with Active Antenna</t>
+          <t>BMP280 Barometric Pressure Sensor</t>
         </is>
       </c>
       <c r="E38" s="3" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="F38" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
     </row>
     <row r="39" ht="20" customHeight="1">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>AI-AIML</t>
+          <t>CCL-AIML</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>AI Project Lab</t>
+          <t>Cloud Computing Lab</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>DEV-JET-02</t>
+          <t>DIS-OLD-01</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>NVIDIA Jetson Orin Nano Developer Kit (8GB)</t>
+          <t>0.96" I2C OLED Display Module (128x64)</t>
         </is>
       </c>
       <c r="E39" s="3" t="n">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
     </row>
     <row r="40" ht="20" customHeight="1">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>AI-AIML</t>
+          <t>MSA-AIML</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>AI Project Lab</t>
+          <t>Multimodal Sensor Analytics Lab</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>ROB-TB3-01</t>
+          <t>SEN-UST-01</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>TurtleBot 3 Burger Mobile Robot</t>
+          <t>Ultrasonic Distance Sensor HC-SR04</t>
         </is>
       </c>
       <c r="E40" s="3" t="n">
+        <v>40</v>
+      </c>
+      <c r="F40" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="F40" s="3" t="n">
-        <v>0</v>
-      </c>
       <c r="G40" s="3" t="n">
-        <v>4</v>
+        <v>44</v>
       </c>
     </row>
     <row r="41" ht="20" customHeight="1">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>AI-AIML</t>
+          <t>MSA-AIML</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>AI Project Lab</t>
+          <t>Multimodal Sensor Analytics Lab</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>CAM-INT-01</t>
+          <t>SEN-DHT-01</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Intel RealSense Depth Camera D435i</t>
+          <t>DHT11 Digital Temperature &amp; Humidity Sensor</t>
         </is>
       </c>
       <c r="E41" s="3" t="n">
-        <v>5</v>
+        <v>35</v>
       </c>
       <c r="F41" s="3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>5</v>
+        <v>37</v>
       </c>
     </row>
     <row r="42" ht="20" customHeight="1">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>AI-AIML</t>
+          <t>MSA-AIML</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>AI Project Lab</t>
+          <t>Multimodal Sensor Analytics Lab</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>OSC-RIG-01</t>
+          <t>SEN-IMU-01</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Rigol DS1054Z 50MHz Digital Oscilloscope</t>
+          <t>MPU6050 6-Axis Gyro &amp; Accelerometer Module</t>
         </is>
       </c>
       <c r="E42" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="F42" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="F42" s="3" t="n">
-        <v>0</v>
-      </c>
       <c r="G42" s="3" t="n">
-        <v>2</v>
+        <v>32</v>
       </c>
     </row>
     <row r="43" ht="20" customHeight="1">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>MIOT-RA</t>
+          <t>MSA-AIML</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Mechatronics and IoT Lab</t>
+          <t>Multimodal Sensor Analytics Lab</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>PLC-SIE-01</t>
+          <t>SEN-BMP-01</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>Siemens SIMATIC S7-1200 CPU 1214C DC/DC/DC</t>
+          <t>BMP280 Barometric Pressure Sensor</t>
         </is>
       </c>
       <c r="E43" s="3" t="n">
-        <v>8</v>
+        <v>25</v>
       </c>
       <c r="F43" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G43" s="3" t="n">
-        <v>8</v>
+        <v>26</v>
       </c>
     </row>
     <row r="44" ht="20" customHeight="1">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>MIOT-RA</t>
+          <t>MSA-AIML</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Mechatronics and IoT Lab</t>
+          <t>Multimodal Sensor Analytics Lab</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>ARM-DOB-01</t>
+          <t>COM-GPS-01</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Dobot Magician 4-DOF Robotic Arm</t>
+          <t>U-Blox Neo-6M GPS Module with Active Antenna</t>
         </is>
       </c>
       <c r="E44" s="3" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="F44" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G44" s="3" t="n">
-        <v>5</v>
+        <v>16</v>
       </c>
     </row>
     <row r="45" ht="20" customHeight="1">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>MIOT-RA</t>
+          <t>MSA-AIML</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Mechatronics and IoT Lab</t>
+          <t>Multimodal Sensor Analytics Lab</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>MOT-SRV-01</t>
+          <t>SEN-PIR-01</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>TowerPro SG90 9g Micro Servo Motor</t>
+          <t>PIR Motion Sensor Module HC-SR501</t>
         </is>
       </c>
       <c r="E45" s="3" t="n">
-        <v>60</v>
+        <v>20</v>
       </c>
       <c r="F45" s="3" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G45" s="3" t="n">
-        <v>65</v>
+        <v>21</v>
       </c>
     </row>
     <row r="46" ht="20" customHeight="1">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>MIOT-RA</t>
+          <t>MSA-AIML</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Mechatronics and IoT Lab</t>
+          <t>Multimodal Sensor Analytics Lab</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>MOT-SRV-02</t>
+          <t>SEN-IRS-01</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>MG996R High Torque Metal Gear Servo Motor</t>
+          <t>Infrared Obstacle Avoidance Sensor Module</t>
         </is>
       </c>
       <c r="E46" s="3" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="F46" s="3" t="n">
         <v>2</v>
       </c>
       <c r="G46" s="3" t="n">
-        <v>32</v>
+        <v>27</v>
       </c>
     </row>
     <row r="47" ht="20" customHeight="1">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>MIOT-RA</t>
+          <t>MSA-AIML</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Mechatronics and IoT Lab</t>
+          <t>Multimodal Sensor Analytics Lab</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>MOT-STP-01</t>
+          <t>SEN-PZO-01</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>NEMA 17 Bipolar Stepper Motor (1.5A 42mm)</t>
+          <t>Piezoelectric Vibration &amp; Knock Sensor</t>
         </is>
       </c>
       <c r="E47" s="3" t="n">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="F47" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G47" s="3" t="n">
-        <v>26</v>
+        <v>16</v>
       </c>
     </row>
     <row r="48" ht="20" customHeight="1">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>MIOT-RA</t>
+          <t>MSA-AIML</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Mechatronics and IoT Lab</t>
+          <t>Multimodal Sensor Analytics Lab</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>DRV-MOT-01</t>
+          <t>DIS-LCD-01</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>L298N Dual H-Bridge Motor Driver Module</t>
+          <t>16x2 Character LCD Display Module</t>
         </is>
       </c>
       <c r="E48" s="3" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="F48" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G48" s="3" t="n">
-        <v>43</v>
+        <v>21</v>
       </c>
     </row>
     <row r="49" ht="20" customHeight="1">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>MIOT-RA</t>
+          <t>AI-AIML</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>Mechatronics and IoT Lab</t>
+          <t>AI Project Lab</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>PWR-LIP-01</t>
+          <t>DEV-JET-02</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>11.1V 3S LiPo Battery Pack 2200mAh 30C</t>
+          <t>NVIDIA Jetson Orin Nano Developer Kit (8GB)</t>
         </is>
       </c>
       <c r="E49" s="3" t="n">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="F49" s="3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G49" s="3" t="n">
-        <v>22</v>
+        <v>8</v>
       </c>
     </row>
     <row r="50" ht="20" customHeight="1">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>MIOT-RA</t>
+          <t>AI-AIML</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Mechatronics and IoT Lab</t>
+          <t>AI Project Lab</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>PWR-ION-01</t>
+          <t>ROB-TB3-01</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>Samsung 18650 Li-ion Cell 3.7V 2600mAh</t>
+          <t>TurtleBot 3 Burger Mobile Robot</t>
         </is>
       </c>
       <c r="E50" s="3" t="n">
-        <v>50</v>
+        <v>4</v>
       </c>
       <c r="F50" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G50" s="3" t="n">
         <v>4</v>
-      </c>
-      <c r="G50" s="3" t="n">
-        <v>54</v>
       </c>
     </row>
     <row r="51" ht="20" customHeight="1">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>MRL-RA</t>
+          <t>AI-AIML</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>Mobile Robotics Lab</t>
+          <t>AI Project Lab</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>ROB-TB3-01</t>
+          <t>CAM-INT-01</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>TurtleBot 3 Burger Mobile Robot</t>
+          <t>Intel RealSense Depth Camera D435i</t>
         </is>
       </c>
       <c r="E51" s="3" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F51" s="3" t="n">
         <v>0</v>
       </c>
       <c r="G51" s="3" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="52" ht="20" customHeight="1">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>MRL-RA</t>
+          <t>AI-AIML</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Mobile Robotics Lab</t>
+          <t>AI Project Lab</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>ROB-TB4-01</t>
+          <t>OSC-RIG-01</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>TurtleBot 4 Standard Mobile Robot</t>
+          <t>Rigol DS1054Z 50MHz Digital Oscilloscope</t>
         </is>
       </c>
       <c r="E52" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F52" s="3" t="n">
         <v>0</v>
       </c>
       <c r="G52" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="53" ht="20" customHeight="1">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>MRL-RA</t>
+          <t>MIOT-RA</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>Mobile Robotics Lab</t>
+          <t>Mechatronics and IoT Lab</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>ARM-KIN-01</t>
+          <t>PLC-SIE-01</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>Kinova Gen3 Lite Robotic Arm</t>
+          <t>Siemens SIMATIC S7-1200 CPU 1214C DC/DC/DC</t>
         </is>
       </c>
       <c r="E53" s="3" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="F53" s="3" t="n">
         <v>0</v>
       </c>
       <c r="G53" s="3" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="54" ht="20" customHeight="1">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>MRL-RA</t>
+          <t>MIOT-RA</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Mobile Robotics Lab</t>
+          <t>Mechatronics and IoT Lab</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>LID-OUS-01</t>
+          <t>ARM-DOB-01</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>Ouster OS1-32 Gen 2 LiDAR Sensor</t>
+          <t>Dobot Magician 4-DOF Robotic Arm</t>
         </is>
       </c>
       <c r="E54" s="3" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F54" s="3" t="n">
         <v>0</v>
       </c>
       <c r="G54" s="3" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="55" ht="20" customHeight="1">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>MRL-RA</t>
+          <t>MIOT-RA</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>Mobile Robotics Lab</t>
+          <t>Mechatronics and IoT Lab</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>SEN-LIN-01</t>
+          <t>MOT-SRV-01</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>TCRT5000 5-Channel Infrared Line Tracking Array</t>
+          <t>TowerPro SG90 9g Micro Servo Motor</t>
         </is>
       </c>
       <c r="E55" s="3" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="F55" s="3" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G55" s="3" t="n">
-        <v>32</v>
+        <v>65</v>
       </c>
     </row>
     <row r="56" ht="20" customHeight="1">
       <c r="A56" s="2" t="inlineStr">
         <is>
+          <t>MIOT-RA</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>Mechatronics and IoT Lab</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>MOT-SRV-02</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>MG996R High Torque Metal Gear Servo Motor</t>
+        </is>
+      </c>
+      <c r="E56" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="F56" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="G56" s="3" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="57" ht="20" customHeight="1">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>MIOT-RA</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>Mechatronics and IoT Lab</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>MOT-STP-01</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>NEMA 17 Bipolar Stepper Motor (1.5A 42mm)</t>
+        </is>
+      </c>
+      <c r="E57" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="F57" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G57" s="3" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="58" ht="20" customHeight="1">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>MIOT-RA</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>Mechatronics and IoT Lab</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>DRV-MOT-01</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>L298N Dual H-Bridge Motor Driver Module</t>
+        </is>
+      </c>
+      <c r="E58" s="3" t="n">
+        <v>40</v>
+      </c>
+      <c r="F58" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="G58" s="3" t="n">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="59" ht="20" customHeight="1">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>MIOT-RA</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>Mechatronics and IoT Lab</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>PWR-LIP-01</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>11.1V 3S LiPo Battery Pack 2200mAh 30C</t>
+        </is>
+      </c>
+      <c r="E59" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="F59" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="G59" s="3" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="60" ht="20" customHeight="1">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>MIOT-RA</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>Mechatronics and IoT Lab</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>PWR-ION-01</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>Samsung 18650 Li-ion Cell 3.7V 2600mAh</t>
+        </is>
+      </c>
+      <c r="E60" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="F60" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="G60" s="3" t="n">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="61" ht="20" customHeight="1">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>MIOT-RA</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>Mechatronics and IoT Lab</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>PWR-9VB-01</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>9V Heavy Duty Alkaline Battery</t>
+        </is>
+      </c>
+      <c r="E61" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="F61" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G61" s="3" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="62" ht="20" customHeight="1">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>MIOT-RA</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>Mechatronics and IoT Lab</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>SEN-PZO-01</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>Piezoelectric Vibration &amp; Knock Sensor</t>
+        </is>
+      </c>
+      <c r="E62" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="F62" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="G62" s="3" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="63" ht="20" customHeight="1">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
           <t>MRL-RA</t>
         </is>
       </c>
-      <c r="B56" s="2" t="inlineStr">
+      <c r="B63" s="2" t="inlineStr">
         <is>
           <t>Mobile Robotics Lab</t>
         </is>
       </c>
-      <c r="C56" s="2" t="inlineStr">
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>ROB-TB3-01</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>TurtleBot 3 Burger Mobile Robot</t>
+        </is>
+      </c>
+      <c r="E63" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="F63" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G63" s="3" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="64" ht="20" customHeight="1">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>MRL-RA</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>Mobile Robotics Lab</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>ROB-TB4-01</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>TurtleBot 4 Standard Mobile Robot</t>
+        </is>
+      </c>
+      <c r="E64" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="F64" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G64" s="3" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="65" ht="20" customHeight="1">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>MRL-RA</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>Mobile Robotics Lab</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>ARM-KIN-01</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>Kinova Gen3 Lite Robotic Arm</t>
+        </is>
+      </c>
+      <c r="E65" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F65" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G65" s="3" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="66" ht="20" customHeight="1">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>MRL-RA</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>Mobile Robotics Lab</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>LID-OUS-01</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>Ouster OS1-32 Gen 2 LiDAR Sensor</t>
+        </is>
+      </c>
+      <c r="E66" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F66" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G66" s="3" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="67" ht="20" customHeight="1">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>MRL-RA</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>Mobile Robotics Lab</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>SEN-LIN-01</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>TCRT5000 5-Channel Infrared Line Tracking Array</t>
+        </is>
+      </c>
+      <c r="E67" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="F67" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="G67" s="3" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="68" ht="20" customHeight="1">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>MRL-RA</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>Mobile Robotics Lab</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
         <is>
           <t>COM-NRF-01</t>
         </is>
       </c>
-      <c r="D56" s="2" t="inlineStr">
+      <c r="D68" s="2" t="inlineStr">
         <is>
           <t>nRF24L01+ 2.4GHz Wireless RF Transceiver</t>
         </is>
       </c>
-      <c r="E56" s="3" t="n">
+      <c r="E68" s="3" t="n">
         <v>40</v>
       </c>
-      <c r="F56" s="3" t="n">
+      <c r="F68" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="G56" s="3" t="n">
+      <c r="G68" s="3" t="n">
         <v>43</v>
       </c>
     </row>
@@ -9727,12 +10334,12 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>WKS-MAC-01</t>
+          <t>MET-DIG-01</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Apple iMac 24" M3 Workstation (16GB / 512GB)</t>
+          <t>Digital Multimeter MAS830L with Test Leads</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -9742,7 +10349,7 @@
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>MAC-261</t>
+          <t>DMM-261</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
@@ -9752,7 +10359,7 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>APL-M3-771101</t>
+          <t>MAS-830-771101</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
@@ -9770,12 +10377,12 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>WKS-MAC-01</t>
+          <t>MET-DIG-01</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Apple iMac 24" M3 Workstation (16GB / 512GB)</t>
+          <t>Digital Multimeter MAS830L with Test Leads</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -9785,7 +10392,7 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>MAC-262</t>
+          <t>DMM-262</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
@@ -9795,7 +10402,7 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>APL-M3-771102</t>
+          <t>MAS-830-771102</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
@@ -9813,12 +10420,12 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>WKS-RTX-01</t>
+          <t>MET-DIG-01</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Dell Precision Tower (NVIDIA RTX 4090 24GB)</t>
+          <t>Digital Multimeter MAS830L with Test Leads</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -9828,7 +10435,7 @@
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>WKS-281</t>
+          <t>DMM-281</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
@@ -9838,7 +10445,7 @@
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>DEL-4090-55101</t>
+          <t>MAS-830-55101</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
@@ -9856,12 +10463,12 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>WKS-RTX-01</t>
+          <t>MET-DIG-01</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Dell Precision Tower (NVIDIA RTX 4090 24GB)</t>
+          <t>Digital Multimeter MAS830L with Test Leads</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -9871,7 +10478,7 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>WKS-282</t>
+          <t>DMM-282</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
@@ -9881,7 +10488,7 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>DEL-4090-55102</t>
+          <t>MAS-830-55102</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">

</xml_diff>

<commit_message>
feat(dcds): complete Phase 03 sealing, DCDS master context reconstruction and full audit log
</commit_message>
<xml_diff>
--- a/public/data/labtrack_master_data.xlsx
+++ b/public/data/labtrack_master_data.xlsx
@@ -4876,7 +4876,7 @@
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="51" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="25" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
     <col width="27" customWidth="1" min="5" max="5"/>
     <col width="83" customWidth="1" min="6" max="6"/>
     <col width="58" customWidth="1" min="7" max="7"/>
@@ -4934,7 +4934,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>DEV-JET-01</t>
+          <t>SBC-JET-01</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -4949,7 +4949,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Microprocessors</t>
+          <t>Single Board Computers</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -4981,7 +4981,7 @@
     <row r="3" ht="20" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>DEV-JET-02</t>
+          <t>SBC-JET-02</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -4996,7 +4996,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Microprocessors</t>
+          <t>Single Board Computers</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -5043,7 +5043,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Microprocessors</t>
+          <t>Single Board Computers</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -5090,7 +5090,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Microprocessors</t>
+          <t>Single Board Computers</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -5231,7 +5231,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Motors</t>
+          <t>Robotics</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -5278,7 +5278,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Motors</t>
+          <t>Robotics</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -5325,7 +5325,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Motors</t>
+          <t>Robotics</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -5372,7 +5372,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Motors</t>
+          <t>Robotics</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -5466,7 +5466,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Misc</t>
+          <t>Actuators</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -5513,7 +5513,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Misc</t>
+          <t>Actuators</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -5607,7 +5607,7 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Misc</t>
+          <t>Actuators</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -6171,7 +6171,7 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Communication Modules</t>
+          <t>Sensors</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -6218,7 +6218,7 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Communication Modules</t>
+          <t>Sensors</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
@@ -6265,7 +6265,7 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Motors</t>
+          <t>Actuators</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
@@ -6312,7 +6312,7 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Motors</t>
+          <t>Actuators</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
@@ -6359,7 +6359,7 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Motors</t>
+          <t>Actuators</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
@@ -6406,7 +6406,7 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Motors</t>
+          <t>Actuators</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
@@ -6453,7 +6453,7 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Batteries</t>
+          <t>Actuators</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
@@ -6500,7 +6500,7 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Batteries</t>
+          <t>Actuators</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
@@ -6547,7 +6547,7 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Batteries</t>
+          <t>Actuators</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
@@ -6594,7 +6594,7 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>Misc</t>
+          <t>Actuators</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
@@ -6641,7 +6641,7 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Misc</t>
+          <t>Actuators</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
@@ -6688,7 +6688,7 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>Misc</t>
+          <t>Actuators</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
@@ -6735,7 +6735,7 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Misc</t>
+          <t>Actuators</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
@@ -7209,12 +7209,12 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>DEV-JET-01</t>
+          <t>SBC-RPI-04</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>NVIDIA Jetson Nano 4GB B01 Developer Kit</t>
+          <t>Raspberry Pi 4 Model B 4GB RAM</t>
         </is>
       </c>
       <c r="E14" s="3" t="n">
@@ -7457,12 +7457,12 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>DEV-JET-02</t>
+          <t>SBC-RPI-05</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>NVIDIA Jetson Orin Nano Developer Kit (8GB)</t>
+          <t>Raspberry Pi 5 Model B 8GB RAM</t>
         </is>
       </c>
       <c r="E22" s="3" t="n">
@@ -7550,7 +7550,7 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>DEV-JET-01</t>
+          <t>SBC-JET-01</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -7705,7 +7705,7 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>DEV-JET-02</t>
+          <t>SBC-JET-02</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -7736,7 +7736,7 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>DEV-JET-01</t>
+          <t>SBC-JET-01</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -7860,7 +7860,7 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>DEV-JET-01</t>
+          <t>SBC-JET-01</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -8294,7 +8294,7 @@
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>DEV-JET-02</t>
+          <t>SBC-JET-02</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
@@ -8912,7 +8912,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I37"/>
+  <dimension ref="A1:I39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -8981,7 +8981,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>DEV-JET-01</t>
+          <t>SBC-JET-01</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -9024,7 +9024,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>DEV-JET-01</t>
+          <t>SBC-JET-01</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -9067,7 +9067,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>DEV-JET-01</t>
+          <t>SBC-JET-01</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -9114,7 +9114,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>DEV-JET-01</t>
+          <t>SBC-JET-01</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -9152,12 +9152,12 @@
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>SIT-CSE-4CL07-0045</t>
+          <t>SIT-AIML-5CL02-0045</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>DEV-JET-01</t>
+          <t>SBC-JET-01</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -9167,7 +9167,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>PL-CSE</t>
+          <t>DV-AIML</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -9195,12 +9195,12 @@
     <row r="7" ht="20" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>SIT-CSE-4CL07-0046</t>
+          <t>SIT-AIML-5CL02-0046</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>DEV-JET-01</t>
+          <t>SBC-JET-01</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -9210,7 +9210,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>PL-CSE</t>
+          <t>DV-AIML</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -9243,7 +9243,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>DEV-JET-02</t>
+          <t>SBC-JET-02</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -9286,7 +9286,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>DEV-JET-02</t>
+          <t>SBC-JET-02</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -9329,7 +9329,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>DEV-JET-02</t>
+          <t>SBC-JET-02</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -9376,7 +9376,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>DEV-JET-02</t>
+          <t>SBC-JET-02</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -9590,37 +9590,37 @@
     <row r="16" ht="20" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>SIT-AIML-5CL03-0101</t>
+          <t>SIT-CSE-5CL01-0085</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>CAM-INT-01</t>
+          <t>SBC-RPI-05</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Intel RealSense Depth Camera D435i</t>
+          <t>Raspberry Pi 5 Model B 8GB RAM</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>CV-AIML</t>
+          <t>MTECH-CSE</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>RS-101</t>
+          <t>RP5-085</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>CPR/2023/0740</t>
+          <t>CPR/2024/0302</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>INT-RS-55210</t>
+          <t>RPI5-8G-002198</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
@@ -9633,37 +9633,37 @@
     <row r="17" ht="20" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>SIT-AIML-5CL03-0102</t>
+          <t>SIT-CSE-4CL07-0086</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>CAM-INT-01</t>
+          <t>SBC-RPI-04</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Intel RealSense Depth Camera D435i</t>
+          <t>Raspberry Pi 4 Model B 4GB RAM</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>CV-AIML</t>
+          <t>PL-CSE</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>RS-102</t>
+          <t>RP4-086</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>CPR/2023/0740</t>
+          <t>CPR/2024/0303</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>INT-RS-55211</t>
+          <t>RPI4-4G-001099</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
@@ -9676,7 +9676,7 @@
     <row r="18" ht="20" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>SIT-AIML-5CL11-0103</t>
+          <t>SIT-AIML-5CL03-0101</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -9691,69 +9691,65 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>AI-AIML</t>
+          <t>CV-AIML</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>RS-103</t>
+          <t>RS-101</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>CPR/2023/0741</t>
+          <t>CPR/2023/0740</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>INT-RS-55212</t>
+          <t>INT-RS-55210</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>IN_USE</t>
-        </is>
-      </c>
-      <c r="I18" s="3" t="inlineStr">
-        <is>
-          <t>25070126076</t>
-        </is>
-      </c>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="n"/>
     </row>
     <row r="19" ht="20" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>SIT-RA-6RA02-0121</t>
+          <t>SIT-AIML-5CL03-0102</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>LID-OUS-01</t>
+          <t>CAM-INT-01</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Ouster OS1-32 Gen 2 LiDAR Sensor</t>
+          <t>Intel RealSense Depth Camera D435i</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>MRL-RA</t>
+          <t>CV-AIML</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>LID-121</t>
+          <t>RS-102</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>CPR/2023/0995</t>
+          <t>CPR/2023/0740</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>OUS-32-11002</t>
+          <t>INT-RS-55211</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
@@ -9766,60 +9762,64 @@
     <row r="20" ht="20" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>SIT-RA-6RA02-0122</t>
+          <t>SIT-AIML-5CL11-0103</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>LID-OUS-01</t>
+          <t>CAM-INT-01</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Ouster OS1-32 Gen 2 LiDAR Sensor</t>
+          <t>Intel RealSense Depth Camera D435i</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>MRL-RA</t>
+          <t>AI-AIML</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>LID-122</t>
+          <t>RS-103</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>CPR/2023/0995</t>
+          <t>CPR/2023/0741</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>OUS-32-11003</t>
+          <t>INT-RS-55212</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>RESERVED</t>
-        </is>
-      </c>
-      <c r="I20" s="2" t="n"/>
+          <t>IN_USE</t>
+        </is>
+      </c>
+      <c r="I20" s="3" t="inlineStr">
+        <is>
+          <t>25070126076</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="20" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>SIT-RA-6RA02-0141</t>
+          <t>SIT-RA-6RA02-0121</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>ROB-TB3-01</t>
+          <t>LID-OUS-01</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>TurtleBot 3 Burger Mobile Robot</t>
+          <t>Ouster OS1-32 Gen 2 LiDAR Sensor</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -9829,17 +9829,17 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>TB3-141</t>
+          <t>LID-121</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>CPR/2024/0410</t>
+          <t>CPR/2023/0995</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>ROB-TB3-77401</t>
+          <t>OUS-32-11002</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
@@ -9852,17 +9852,17 @@
     <row r="22" ht="20" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>SIT-RA-6RA02-0142</t>
+          <t>SIT-RA-6RA02-0122</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>ROB-TB3-01</t>
+          <t>LID-OUS-01</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>TurtleBot 3 Burger Mobile Robot</t>
+          <t>Ouster OS1-32 Gen 2 LiDAR Sensor</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -9872,22 +9872,22 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>TB3-142</t>
+          <t>LID-122</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>CPR/2024/0410</t>
+          <t>CPR/2023/0995</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>ROB-TB3-77402</t>
+          <t>OUS-32-11003</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>AVAILABLE</t>
+          <t>RESERVED</t>
         </is>
       </c>
       <c r="I22" s="2" t="n"/>
@@ -9895,7 +9895,7 @@
     <row r="23" ht="20" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>SIT-AIML-5CL11-0143</t>
+          <t>SIT-RA-6RA02-0141</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -9910,49 +9910,45 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>AI-AIML</t>
+          <t>MRL-RA</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>TB3-143</t>
+          <t>TB3-141</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>CPR/2024/0411</t>
+          <t>CPR/2024/0410</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>ROB-TB3-77403</t>
+          <t>ROB-TB3-77401</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>IN_USE</t>
-        </is>
-      </c>
-      <c r="I23" s="3" t="inlineStr">
-        <is>
-          <t>24070127008</t>
-        </is>
-      </c>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="n"/>
     </row>
     <row r="24" ht="20" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>SIT-RA-6RA02-0161</t>
+          <t>SIT-RA-6RA02-0142</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>ROB-TB4-01</t>
+          <t>ROB-TB3-01</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>TurtleBot 4 Standard Mobile Robot</t>
+          <t>TurtleBot 3 Burger Mobile Robot</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -9962,17 +9958,17 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>TB4-161</t>
+          <t>TB3-142</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>CPR/2024/1205</t>
+          <t>CPR/2024/0410</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>CP-TB4-00109</t>
+          <t>ROB-TB3-77402</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
@@ -9985,80 +9981,84 @@
     <row r="25" ht="20" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>SIT-RA-6RA02-0162</t>
+          <t>SIT-AIML-5CL11-0143</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>ROB-TB4-01</t>
+          <t>ROB-TB3-01</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>TurtleBot 4 Standard Mobile Robot</t>
+          <t>TurtleBot 3 Burger Mobile Robot</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>MRL-RA</t>
+          <t>AI-AIML</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>TB4-162</t>
+          <t>TB3-143</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>CPR/2024/1205</t>
+          <t>CPR/2024/0411</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>CP-TB4-00110</t>
+          <t>ROB-TB3-77403</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>AVAILABLE</t>
-        </is>
-      </c>
-      <c r="I25" s="2" t="n"/>
+          <t>IN_USE</t>
+        </is>
+      </c>
+      <c r="I25" s="3" t="inlineStr">
+        <is>
+          <t>24070127008</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="20" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>SIT-RA-6RA01-0181</t>
+          <t>SIT-RA-6RA02-0161</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>ARM-DOB-01</t>
+          <t>ROB-TB4-01</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Dobot Magician 4-DOF Robotic Arm</t>
+          <t>TurtleBot 4 Standard Mobile Robot</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>MIOT-RA</t>
+          <t>MRL-RA</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>DOB-181</t>
+          <t>TB4-161</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>CPR/2023/1080</t>
+          <t>CPR/2024/1205</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>DOB-MAG-33901</t>
+          <t>CP-TB4-00109</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
@@ -10071,37 +10071,37 @@
     <row r="27" ht="20" customHeight="1">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>SIT-RA-6RA01-0182</t>
+          <t>SIT-RA-6RA02-0162</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>ARM-DOB-01</t>
+          <t>ROB-TB4-01</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Dobot Magician 4-DOF Robotic Arm</t>
+          <t>TurtleBot 4 Standard Mobile Robot</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>MIOT-RA</t>
+          <t>MRL-RA</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>DOB-182</t>
+          <t>TB4-162</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>CPR/2023/1080</t>
+          <t>CPR/2024/1205</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>DOB-MAG-33902</t>
+          <t>CP-TB4-00110</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
@@ -10114,37 +10114,37 @@
     <row r="28" ht="20" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>SIT-RA-6RA02-0201</t>
+          <t>SIT-RA-6RA01-0181</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>ARM-KIN-01</t>
+          <t>ARM-DOB-01</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Kinova Gen3 Lite Robotic Arm</t>
+          <t>Dobot Magician 4-DOF Robotic Arm</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>MRL-RA</t>
+          <t>MIOT-RA</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>KIN-201</t>
+          <t>DOB-181</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>CPR/2023/1350</t>
+          <t>CPR/2023/1080</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>KIN-G3L-00441</t>
+          <t>DOB-MAG-33901</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
@@ -10157,17 +10157,17 @@
     <row r="29" ht="20" customHeight="1">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>SIT-RA-6RA01-0221</t>
+          <t>SIT-RA-6RA01-0182</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>PLC-SIE-01</t>
+          <t>ARM-DOB-01</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Siemens SIMATIC S7-1200 CPU 1214C DC/DC/DC</t>
+          <t>Dobot Magician 4-DOF Robotic Arm</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
@@ -10177,17 +10177,17 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>PLC-221</t>
+          <t>DOB-182</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>CPR/2023/0620</t>
+          <t>CPR/2023/1080</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>SIE-S7-882101</t>
+          <t>DOB-MAG-33902</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -10200,37 +10200,37 @@
     <row r="30" ht="20" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>SIT-RA-6RA01-0222</t>
+          <t>SIT-RA-6RA02-0201</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>PLC-SIE-01</t>
+          <t>ARM-KIN-01</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Siemens SIMATIC S7-1200 CPU 1214C DC/DC/DC</t>
+          <t>Kinova Gen3 Lite Robotic Arm</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>MIOT-RA</t>
+          <t>MRL-RA</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>PLC-222</t>
+          <t>KIN-201</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>CPR/2023/0620</t>
+          <t>CPR/2023/1350</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>SIE-S7-882102</t>
+          <t>KIN-G3L-00441</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -10243,37 +10243,37 @@
     <row r="31" ht="20" customHeight="1">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>SIT-CSE-4CL07-0241</t>
+          <t>SIT-RA-6RA01-0221</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>OSC-RIG-01</t>
+          <t>PLC-SIE-01</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Rigol DS1054Z 50MHz Digital Oscilloscope</t>
+          <t>Siemens SIMATIC S7-1200 CPU 1214C DC/DC/DC</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>PL-CSE</t>
+          <t>MIOT-RA</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>OSC-241</t>
+          <t>PLC-221</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>CPR/2022/1501</t>
+          <t>CPR/2023/0620</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>RIG-DS-99104</t>
+          <t>SIE-S7-882101</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
@@ -10286,37 +10286,37 @@
     <row r="32" ht="20" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>SIT-AIML-5CL11-0242</t>
+          <t>SIT-RA-6RA01-0222</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>OSC-RIG-01</t>
+          <t>PLC-SIE-01</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Rigol DS1054Z 50MHz Digital Oscilloscope</t>
+          <t>Siemens SIMATIC S7-1200 CPU 1214C DC/DC/DC</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>AI-AIML</t>
+          <t>MIOT-RA</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>OSC-242</t>
+          <t>PLC-222</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>CPR/2022/1502</t>
+          <t>CPR/2023/0620</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>RIG-DS-99105</t>
+          <t>SIE-S7-882102</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
@@ -10329,37 +10329,37 @@
     <row r="33" ht="20" customHeight="1">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>SIT-AIML-5CL03-0261</t>
+          <t>SIT-CSE-4CL07-0241</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>MET-DIG-01</t>
+          <t>OSC-RIG-01</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Digital Multimeter MAS830L with Test Leads</t>
+          <t>Rigol DS1054Z 50MHz Digital Oscilloscope</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>CV-AIML</t>
+          <t>PL-CSE</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>DMM-261</t>
+          <t>OSC-241</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>CPR/2024/0115</t>
+          <t>CPR/2022/1501</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>MAS-830-771101</t>
+          <t>RIG-DS-99104</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
@@ -10372,37 +10372,37 @@
     <row r="34" ht="20" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>SIT-AIML-5CL03-0262</t>
+          <t>SIT-AIML-5CL11-0242</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>MET-DIG-01</t>
+          <t>OSC-RIG-01</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Digital Multimeter MAS830L with Test Leads</t>
+          <t>Rigol DS1054Z 50MHz Digital Oscilloscope</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>CV-AIML</t>
+          <t>AI-AIML</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>DMM-262</t>
+          <t>OSC-242</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>CPR/2024/0115</t>
+          <t>CPR/2022/1502</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>MAS-830-771102</t>
+          <t>RIG-DS-99105</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
@@ -10415,7 +10415,7 @@
     <row r="35" ht="20" customHeight="1">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>SIT-AIML-5CL02-0281</t>
+          <t>SIT-AIML-5CL03-0261</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
@@ -10430,22 +10430,22 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>DV-AIML</t>
+          <t>CV-AIML</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>DMM-281</t>
+          <t>DMM-261</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>CPR/2024/0220</t>
+          <t>CPR/2024/0115</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>MAS-830-55101</t>
+          <t>MAS-830-771101</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
@@ -10458,7 +10458,7 @@
     <row r="36" ht="20" customHeight="1">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>SIT-CSE-5CL01-0282</t>
+          <t>SIT-AIML-5CL03-0262</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -10473,22 +10473,22 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>MTECH-CSE</t>
+          <t>CV-AIML</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>DMM-282</t>
+          <t>DMM-262</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>CPR/2024/0220</t>
+          <t>CPR/2024/0115</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>MAS-830-55102</t>
+          <t>MAS-830-771102</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
@@ -10501,45 +10501,131 @@
     <row r="37" ht="20" customHeight="1">
       <c r="A37" s="2" t="inlineStr">
         <is>
+          <t>SIT-AIML-5CL02-0281</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>MET-DIG-01</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>Digital Multimeter MAS830L with Test Leads</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>DV-AIML</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>DMM-281</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>CPR/2024/0220</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>MAS-830-55101</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="n"/>
+    </row>
+    <row r="38" ht="20" customHeight="1">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>SIT-CSE-5CL01-0282</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>MET-DIG-01</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>Digital Multimeter MAS830L with Test Leads</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>MTECH-CSE</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>DMM-282</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>CPR/2024/0220</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>MAS-830-55102</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>AVAILABLE</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="n"/>
+    </row>
+    <row r="39" ht="20" customHeight="1">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
           <t>SIT-AIML-5CL03-0301</t>
         </is>
       </c>
-      <c r="B37" s="2" t="inlineStr">
+      <c r="B39" s="2" t="inlineStr">
         <is>
           <t>CAM-FLI-01</t>
         </is>
       </c>
-      <c r="C37" s="2" t="inlineStr">
+      <c r="C39" s="2" t="inlineStr">
         <is>
           <t>FLIR Lepton 3.5 Radiometric LWIR Thermal Camera</t>
         </is>
       </c>
-      <c r="D37" s="2" t="inlineStr">
+      <c r="D39" s="2" t="inlineStr">
         <is>
           <t>CV-AIML</t>
         </is>
       </c>
-      <c r="E37" s="2" t="inlineStr">
+      <c r="E39" s="2" t="inlineStr">
         <is>
           <t>FLI-301</t>
         </is>
       </c>
-      <c r="F37" s="2" t="inlineStr">
+      <c r="F39" s="2" t="inlineStr">
         <is>
           <t>CPR/2023/1188</t>
         </is>
       </c>
-      <c r="G37" s="2" t="inlineStr">
+      <c r="G39" s="2" t="inlineStr">
         <is>
           <t>FLI-LEP-22019</t>
         </is>
       </c>
-      <c r="H37" s="2" t="inlineStr">
+      <c r="H39" s="2" t="inlineStr">
         <is>
           <t>AVAILABLE</t>
         </is>
       </c>
-      <c r="I37" s="2" t="n"/>
+      <c r="I39" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -10954,7 +11040,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D23"/>
+  <dimension ref="A1:D24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -11274,22 +11360,22 @@
     <row r="15" ht="20" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>PROJ-000005</t>
+          <t>PROJ-000004</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>24070127008</t>
+          <t>25070126076</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Kunal Gokhale</t>
+          <t>Ishaan Chand</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>LEAD</t>
+          <t>COLLABORATOR</t>
         </is>
       </c>
     </row>
@@ -11301,17 +11387,17 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>24070127021</t>
+          <t>24070127008</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Ritika Roy</t>
+          <t>Kunal Gokhale</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>MEMBER</t>
+          <t>LEAD</t>
         </is>
       </c>
     </row>
@@ -11323,12 +11409,12 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>24070127035</t>
+          <t>24070127021</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Tushar Agrawal</t>
+          <t>Ritika Roy</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -11340,22 +11426,22 @@
     <row r="18" ht="20" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>PROJ-000006</t>
+          <t>PROJ-000005</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>24070122009</t>
+          <t>24070127035</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Siddharth Menon</t>
+          <t>Tushar Agrawal</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>LEAD</t>
+          <t>MEMBER</t>
         </is>
       </c>
     </row>
@@ -11367,39 +11453,39 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>24070122022</t>
+          <t>24070122009</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Kavya Iyer</t>
+          <t>Siddharth Menon</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>MEMBER</t>
+          <t>LEAD</t>
         </is>
       </c>
     </row>
     <row r="20" ht="20" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>PROJ-000007</t>
+          <t>PROJ-000006</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>23070126012</t>
+          <t>24070122022</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Aryan Saxena</t>
+          <t>Kavya Iyer</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>LEAD</t>
+          <t>MEMBER</t>
         </is>
       </c>
     </row>
@@ -11411,39 +11497,39 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>23070126025</t>
+          <t>23070126012</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Sneha Kulkarni</t>
+          <t>Aryan Saxena</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>MEMBER</t>
+          <t>LEAD</t>
         </is>
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>PROJ-000008</t>
+          <t>PROJ-000007</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>23070127014</t>
+          <t>23070126025</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Deepak Solanki</t>
+          <t>Sneha Kulkarni</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>LEAD</t>
+          <t>MEMBER</t>
         </is>
       </c>
     </row>
@@ -11455,15 +11541,37 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
+          <t>23070127014</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Deepak Solanki</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>LEAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>PROJ-000008</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
           <t>23070127027</t>
         </is>
       </c>
-      <c r="C23" s="2" t="inlineStr">
+      <c r="C24" s="2" t="inlineStr">
         <is>
           <t>Aishwarya Mane</t>
         </is>
       </c>
-      <c r="D23" s="2" t="inlineStr">
+      <c r="D24" s="2" t="inlineStr">
         <is>
           <t>MEMBER</t>
         </is>

</xml_diff>